<commit_message>
Padroniza atualizacao das planilhas
</commit_message>
<xml_diff>
--- a/EAP_PRODUCAO.xlsx
+++ b/EAP_PRODUCAO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72C358BF-8DF4-4D62-BADE-D5393D7E8BF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AA540C8-E5A2-40B7-9983-66D5BB8B77CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -953,7 +953,7 @@
         <v>2426.84</v>
       </c>
       <c r="E16" s="2">
-        <v>1538.59</v>
+        <v>1460.1</v>
       </c>
       <c r="F16">
         <v>2735</v>
@@ -963,7 +963,7 @@
       </c>
       <c r="I16" s="5">
         <f t="shared" si="0"/>
-        <v>888.25000000000023</v>
+        <v>966.74000000000024</v>
       </c>
       <c r="J16" s="5"/>
     </row>
@@ -1109,19 +1109,19 @@
     <row r="27" spans="2:16" x14ac:dyDescent="0.3">
       <c r="P27">
         <f>SUM(E3:E16)</f>
-        <v>15410.495000000003</v>
+        <v>15332.005000000003</v>
       </c>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.3">
       <c r="P28">
         <f>14468.56-P27</f>
-        <v>-941.93500000000313</v>
+        <v>-863.44500000000335</v>
       </c>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.3">
       <c r="P29">
         <f>P28+2135.09</f>
-        <v>1193.154999999997</v>
+        <v>1271.6449999999968</v>
       </c>
     </row>
     <row r="34" spans="8:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza PDS e planos Joao Canzi
</commit_message>
<xml_diff>
--- a/EAP_PRODUCAO.xlsx
+++ b/EAP_PRODUCAO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C64D580-29E9-40FC-91FE-F87705B4D0F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4F77330-4780-48E6-88FD-AC6520BEC045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -978,8 +978,8 @@
         <v>2545.85</v>
       </c>
       <c r="E17" s="2">
-        <f>487.87+84.32+43.66</f>
-        <v>615.85</v>
+        <f>487.87+84.32+43.66+62.701</f>
+        <v>678.55100000000004</v>
       </c>
       <c r="F17">
         <v>2361</v>
@@ -989,7 +989,7 @@
       </c>
       <c r="I17" s="5">
         <f t="shared" si="0"/>
-        <v>1930</v>
+        <v>1867.299</v>
       </c>
     </row>
     <row r="18" spans="2:16" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza PDS e mapa 2026-05-25
</commit_message>
<xml_diff>
--- a/EAP_PRODUCAO.xlsx
+++ b/EAP_PRODUCAO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4F77330-4780-48E6-88FD-AC6520BEC045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{756AE521-D5AA-4E0D-B1B2-BE7BDE482BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -978,8 +978,8 @@
         <v>2545.85</v>
       </c>
       <c r="E17" s="2">
-        <f>487.87+84.32+43.66+62.701</f>
-        <v>678.55100000000004</v>
+        <f>487.87+84.32+43.66+62.701+80.157</f>
+        <v>758.70800000000008</v>
       </c>
       <c r="F17">
         <v>2361</v>
@@ -989,7 +989,7 @@
       </c>
       <c r="I17" s="5">
         <f t="shared" si="0"/>
-        <v>1867.299</v>
+        <v>1787.1419999999998</v>
       </c>
     </row>
     <row r="18" spans="2:16" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza EAP com TL0 recebidas
</commit_message>
<xml_diff>
--- a/EAP_PRODUCAO.xlsx
+++ b/EAP_PRODUCAO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8900B8A9-2E78-44B9-AE67-C4ABEB1DF9BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C08B53EA-FE7F-4BCD-AF06-F035C77144C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="21">
   <si>
     <t>Ano</t>
   </si>
@@ -93,6 +93,9 @@
   </si>
   <si>
     <t>mar de coral esta com o valor de as built</t>
+  </si>
+  <si>
+    <t>TL-0 Recebidas</t>
   </si>
 </sst>
 </file>
@@ -590,6 +593,7 @@
     <col min="5" max="5" width="13.21875" customWidth="1"/>
     <col min="6" max="6" width="15.77734375" customWidth="1"/>
     <col min="7" max="7" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.109375" customWidth="1"/>
     <col min="9" max="10" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
@@ -613,6 +617,9 @@
       <c r="G2" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="H2" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="3" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B3" s="2">
@@ -984,7 +991,10 @@
         <v>2361</v>
       </c>
       <c r="G17">
-        <v>0</v>
+        <v>87</v>
+      </c>
+      <c r="H17">
+        <v>189</v>
       </c>
       <c r="I17" s="5">
         <f t="shared" si="0"/>

</xml_diff>

<commit_message>
Atualiza extensao e EAP
</commit_message>
<xml_diff>
--- a/EAP_PRODUCAO.xlsx
+++ b/EAP_PRODUCAO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95249EB5-ECF0-408A-BCF3-3BA976DCDBCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{582B2045-271D-44A5-AD11-CD06CF7902B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_PRODUCAO" sheetId="2" r:id="rId1"/>
@@ -729,7 +729,7 @@
         <v>584</v>
       </c>
       <c r="I7" s="5">
-        <f t="shared" ref="I7:I18" si="0">D7-E7</f>
+        <f t="shared" ref="I7:I19" si="0">D7-E7</f>
         <v>-473.39499999999998</v>
       </c>
       <c r="J7" s="5"/>
@@ -1035,11 +1035,18 @@
       <c r="D19" s="3">
         <v>3269.49</v>
       </c>
+      <c r="E19" s="2">
+        <v>405.2</v>
+      </c>
       <c r="F19">
         <v>4487</v>
       </c>
       <c r="G19">
         <v>0</v>
+      </c>
+      <c r="I19" s="5">
+        <f t="shared" si="0"/>
+        <v>2864.29</v>
       </c>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza EAP extensao e PDS de 13 julho
</commit_message>
<xml_diff>
--- a/EAP_PRODUCAO.xlsx
+++ b/EAP_PRODUCAO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46264610-EC5E-4720-890F-4D3F5AF98960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4326D0D5-AA73-4B57-8975-2617567A25D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1036,7 +1036,7 @@
         <v>3269.49</v>
       </c>
       <c r="E19" s="2">
-        <v>439.7</v>
+        <v>753.5</v>
       </c>
       <c r="F19">
         <v>4487</v>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="I19" s="5">
         <f t="shared" si="0"/>
-        <v>2829.79</v>
+        <v>2515.9899999999998</v>
       </c>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.3">

</xml_diff>